<commit_message>
Regenera registos SGQ/SGA/SGE e corrige build SGE para a IM-009
O build SGE falhava com KeyError em edata.campanha(): a IM-009 entrou em
dimse.py com a tecnologia "Injetora totalmente elétrica (linha dedicada a
contacto alimentar)". Nas injetoras, o fator kW passa a usar a tecnologia
sem a nota entre parênteses; o rótulo completo mantém-se nos registos.
As ISBM continuam com correspondência exata ("ISBM híbrida (servo)").

Registos SGQ (20), SGA (22) e SGE (15) regenerados com os scripts _build
atualizados; 0 erros de fórmula nos três sistemas.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SGI_Sistema-de-gestao-integrado/SGA_Sistema-de-gestao-ambiental/Registos_SGA_Plasticom/SGA-00_Indice_Modelo_Dados.xlsx
+++ b/SGI_Sistema-de-gestao-integrado/SGA_Sistema-de-gestao-ambiental/Registos_SGA_Plasticom/SGA-00_Indice_Modelo_Dados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Project Portfolios\manufacturing-performance-analytics\SGI_Sistema-de-gestao-integrado\SGA_Sistema-de-gestao-ambiental\Registos_SGA_Plasticom\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A7DF4F5-66ED-4BAB-9DA7-8AF7A73E040D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3FE8D9F-7B4A-46E7-97D1-6B93513DA752}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1920" yWindow="1920" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3192,7 +3192,7 @@
     <t>Produtivo</t>
   </si>
   <si>
-    <t>IM-001 a IM-008</t>
+    <t>IM-001 a IM-009</t>
   </si>
   <si>
     <t>SOP</t>

</xml_diff>